<commit_message>
Trim RTI to capture and copilot: remove in-app analysis
House captures, makes recallable, and assists in the moment. Analysis moves
downstream to the vault and Pi.

Removed: live Notes, Discussion Guide and Findings (tabs, controllers,
prompts, settings, guide context in Assist), the end-of-session summary and
generated title, the summary-ready notification, the Session summary action,
the saved-meeting outputs (recipes, templates, chooser), Edit and Regenerate
Summary, and the offline prompt lab.

Kept: recording, live transcript, screenshots, session archive, automatic
transcript upgrade, vault router and /meeting trigger, Sessions window,
Auto mode, Recap, listener actions, the rest of the copilot.

Phase summarizing is now upgrading; the record control and control socket say
Session saved and Upgrading transcript.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VydPNw8QreBBTMDGVc2fsn
</commit_message>
<xml_diff>
--- a/docs/rti_feature_tracker.xlsx
+++ b/docs/rti_feature_tracker.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K75"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to open the Setup tab from the overlay chrome so I can configure project context, live panels, and discussion guides before recording.</t>
+          <t>As a user, I want to open the Setup tab from the overlay chrome so I can configure project context and live aids before recording.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Start transitions idle or done into a fresh live session; stop finalizes capture, runs archive and summary flows, and blocks restart during finishing.</t>
+          <t>Start transitions idle or done into a fresh live session; stop finalizes capture, runs archive and transcript upgrade flows, and blocks restart during finishing.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1828,27 +1828,27 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>DGU-001</t>
+          <t>ANA-005</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Discussion guide import from project vault</t>
+          <t>Enable Auto live analysis</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to discover discussion guides already attached to the selected project.</t>
+          <t>As a user, I want RTI to proactively surface suggestions only when I opt into that behavior.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>When the chosen workstream is a project, Setup lists guide files found in that project and allows loading them into the parser preview.</t>
+          <t>Auto is opt-in, appears as a live panel toggle, and when enabled schedules proactive card generation plus quiet-window debounced generation after speech settles.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Session/VaultWorkstreamStore.swift</t>
+          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Session/SessionCoordinator.swift; RTI/Sources/Analysis/AutoAssistController.swift</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1877,37 +1877,37 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>DGU-002</t>
+          <t>ANA-006</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Discussion guide paste and upload</t>
+          <t>Auto tab suggestions</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to add a discussion guide from pasted text or an uploaded file.</t>
+          <t>As a user, I want live proactive suggestions about what to say, ask, recall, or flag.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Setup supports pasted guide text plus upload of markdown, text, docx, doc, pdf, rtf, and html sources, extracting text and parsing it into a preview.</t>
+          <t>The Auto tab shows SAY, ASK, RECALL, and FLAG cards, manual resurface, copy support, and unseen-count semantics when the user has not viewed the tab.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Setup</t>
+          <t>Overlay &gt; Auto</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Analysis/DiscussionGuideController.swift; RTI/Sources/Analysis/GuideTextExtractor.swift</t>
+          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Analysis/AutoAssistController.swift</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1926,37 +1926,37 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>DGU-003</t>
+          <t>AST-001</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Discussion guide preview and confirmation</t>
+          <t>Freeform ask-anything composer</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to preview the parsed guide before it becomes active so I can catch parser mistakes.</t>
+          <t>As a user, I want to type my own question to RTI instead of relying only on canned actions.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Parsed guides become pending first, showing objective and section structure; the user can confirm, discard, or later remove the active guide.</t>
+          <t>The overlay composer accepts freeform text, submits on Return, clears draft on session stop, and routes the text through the standard LLM pipeline.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Setup</t>
+          <t>Overlay composer</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Analysis/DiscussionGuideController.swift</t>
+          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1975,37 +1975,37 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>DGU-004</t>
+          <t>AST-002</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Guide</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Live guide coverage tab</t>
+          <t>Assist quick action</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to show which discussion-guide questions have been answered during the meeting.</t>
+          <t>As a user, I want RTI to suggest what I should say next.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>If a guide is active, the Guide tab shows coverage stats and structured objective sections; otherwise it shows an empty state instructing the user to attach a guide from Setup.</t>
+          <t>The Assist action sends the current prompt-store Assist prompt, grounded in recent transcript and meeting context, and streams a response into the chat.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Guide</t>
+          <t>Overlay actions menu; Command-Return; command palette</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Analysis/DiscussionGuideController.swift</t>
+          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2024,37 +2024,37 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ANA-001</t>
+          <t>AST-003</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Enable Notes live analysis</t>
+          <t>Say Next quick action</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to turn Notes on only when I need it so the extra live analysis stays opt-in.</t>
+          <t>As a user, I want a terse one-line draft reply.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Notes is off by default, becomes available as a live panel toggle, and when enabled adds the Notes tab and lets the scheduler generate note batches during the session.</t>
+          <t>The Say Next action is available as a quick action and global hotkey and requests a one-line reply through the assistant pipeline.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Setup; Settings &gt; General</t>
+          <t>Overlay actions menu; Command-Option-S</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
+          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2073,37 +2073,37 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ANA-002</t>
+          <t>AST-004</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Notes tab controls</t>
+          <t>Follow-up Questions quick action</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to manually regenerate, copy, and export generated notes.</t>
+          <t>As a user, I want RTI to propose follow-up questions based on the conversation.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>The Notes tab shows progress, errors, note blocks with time ranges, copy-per-block, copy-all, regenerate-now, and export-to-markdown actions.</t>
+          <t>The Follow-ups action uses its prompt-store prompt, and streams results in chat.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Notes</t>
+          <t>Overlay actions menu; Command-Option-F</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Analysis/NotesGenerationController.swift</t>
+          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2122,37 +2122,37 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ANA-003</t>
+          <t>AST-005</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Enable Findings live analysis</t>
+          <t>Recap quick action and recap depth</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to turn the Findings ledger on when I want a running list of tensions and missed threads.</t>
+          <t>As a user, I want fast recaps at different levels of detail.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Findings is opt-in, appears as a live panel toggle, and when enabled adds a Findings tab backed by scheduled generation.</t>
+          <t>RTI offers Recap as an action, persists a sticky recap depth, and also supports brief and detailed one-shot recap variants via commands.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Setup</t>
+          <t>Overlay actions menu; Command-Option-R; command palette</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Session/SessionCoordinator.swift; RTI/Sources/Analysis/FindingsController.swift</t>
+          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2162,50 +2162,46 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>passed-manual</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>Manual check on 2026-06-30: toggling Findings on immediately added the Findings tab; toggling it back off removed the tab.</t>
-        </is>
-      </c>
+      <c r="K34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ANA-004</t>
+          <t>AST-007</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Findings tab controls</t>
+          <t>Listener-mode research actions</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to inspect, copy, and export tagged findings during a call.</t>
+          <t>As a passive observer, I want RTI to switch from speaking advice to observation-centric research prompts.</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>The Findings tab shows tagged entries with timestamps, optional quotes and speakers, manual rescan, copy-per-entry, copy-all, and markdown export.</t>
+          <t>Listener mode exposes Key Tensions, What's Unsaid or Probe, and Emerging Themes actions and adjusts Assist and Follow-ups framing for observer sessions.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Findings</t>
+          <t>Overlay actions menu; command palette; hotkeys</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Analysis/FindingsController.swift</t>
+          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2224,37 +2220,37 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ANA-005</t>
+          <t>AST-008</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Enable Auto live analysis</t>
+          <t>Primary action remap</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to proactively surface suggestions only when I opt into that behavior.</t>
+          <t>As a user, I want Command-Return to run the quick action I use most.</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Auto is opt-in, appears as a live panel toggle, and when enabled schedules proactive card generation plus quiet-window debounced generation after speech settles.</t>
+          <t>The primary action can be remapped to any eligible assistant action, persists in user defaults, and is reflected in the actions menu and command surfaces.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Setup</t>
+          <t>Overlay actions menu; menu</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Session/SessionCoordinator.swift; RTI/Sources/Analysis/AutoAssistController.swift</t>
+          <t>RTI/Sources/LLM/LLMController.swift; RTI/Core/LLM/AssistantAction.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2273,37 +2269,37 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ANA-006</t>
+          <t>AST-009</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Auto tab suggestions</t>
+          <t>Smart mode toggle</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want live proactive suggestions about what to say, ask, recall, or flag.</t>
+          <t>As a user, I want to toggle reasoning-heavy responses when the extra latency is worth it.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>The Auto tab shows SAY, ASK, RECALL, and FLAG cards, manual resurface, copy support, and unseen-count semantics when the user has not viewed the tab.</t>
+          <t>Smart mode persists to user defaults and flips the LLM pipeline into smart-mode requests unless a given action already forces smart behavior.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Auto</t>
+          <t>Menu; command palette; overlay actions menu indicator</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Analysis/AutoAssistController.swift</t>
+          <t>RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2322,7 +2318,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AST-001</t>
+          <t>AST-010</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2332,27 +2328,27 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Freeform ask-anything composer</t>
+          <t>Clear current chat</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to type my own question to RTI instead of relying only on canned actions.</t>
+          <t>As a user, I want to wipe the current chat transcript without touching the live meeting transcript.</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>The overlay composer accepts freeform text, submits on Return, clears draft on session stop, and routes the text through the standard LLM pipeline.</t>
+          <t>Clearing chat cancels any in-flight stream, removes in-memory assistant entries immediately, and hides auxiliary floating panels without a confirmation modal.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Overlay composer</t>
+          <t>Menu; overlay more menu; command palette</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/AppDelegate.swift; RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2371,7 +2367,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AST-002</t>
+          <t>AST-011</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2381,27 +2377,27 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Assist quick action</t>
+          <t>Streaming status and cancellation</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to suggest what I should say next.</t>
+          <t>As a user, I want to see when RTI is still thinking or using a tool and stop it if needed.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>The Assist action sends the current prompt-store Assist prompt, grounded in recent transcript and meeting context, and streams a response into the chat.</t>
+          <t>While a response streams, the chat tracks streaming and reasoning state plus tool status; the composer swaps send for stop and cancellation prunes empty assistant output.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; Command-Return; command palette</t>
+          <t>Overlay chat</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2420,7 +2416,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AST-003</t>
+          <t>AST-012</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2430,27 +2426,27 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Say Next quick action</t>
+          <t>Assistant provider hot swap</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want a terse one-line draft reply.</t>
+          <t>As a user, I want to switch LLM providers without restarting RTI so the next assistant turn uses a different backend immediately.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>The Say Next action is available as a quick action and global hotkey and requests a one-line reply through the assistant pipeline.</t>
+          <t>Assistant provider selection persists, is exposed in Providers settings plus menu and overlay quick-switch surfaces, and the next LLM request resolves the newly active provider at call time.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; Command-Option-S</t>
+          <t>Settings &gt; Providers; menu; overlay more menu</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/LLM/LLMProvider.swift; RTI/Sources/LLM/LLMClient.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2460,16 +2456,20 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>passed-manual</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Overlay More-actions menu shows Assistant provider and Transcription provider submenus on fresh app process 2026-06-30.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>AST-004</t>
+          <t>AST-013</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2479,27 +2479,27 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Follow-up Questions quick action</t>
+          <t>Quick note insertion mode</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to propose follow-up questions based on the conversation.</t>
+          <t>As a user, I want to flip between normal chat and a quick note insert mode with almost no friction.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>The Follow-ups action uses its prompt-store prompt, includes guide coverage context when present, and streams results in chat.</t>
+          <t>The Assist composer shows a visible `Chat`/`Note` toggle during a live session, keeps focus in the field when toggled, inserts note text inline into the transcript on Enter, and then returns to chat mode automatically for one-off notes.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; Command-Option-F</t>
+          <t>Overlay composer</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Sources/UI/Overlay/OverlayInputState.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2509,46 +2509,50 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>automated-pass</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>UX change implemented 2026-06-30; manual pass still pending.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>AST-005</t>
+          <t>SCR-001</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Screenshot</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Recap quick action and recap depth</t>
+          <t>Context capture by hotkey or menu</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want fast recaps at different levels of detail.</t>
+          <t>As a user, I want to attach OCR from the current screen to my next assistant turn.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>RTI offers Recap as an action, persists a sticky recap depth, and also supports brief and detailed one-shot recap variants via commands.</t>
+          <t>Capture Screen runs from command surfaces, uses screenshot plus OCR services, and stores extracted text as pending screen context for the next LLM message rather than sending raw images to the model.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; Command-Option-R; command palette</t>
+          <t>Command-Shift-H; overlay more menu; command palette</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
+          <t>RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/Screenshot/ScreenshotManager.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2567,37 +2571,37 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>AST-006</t>
+          <t>SCR-002</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Screenshot</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Session summary quick action</t>
+          <t>Image drag-and-drop OCR</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to generate a full meeting summary over the complete transcript so far.</t>
+          <t>As a user, I want to drop an image onto the composer to extract text into the next message.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>The Session Summary action forces the smart model and runs over the full transcript window rather than the recent context slice.</t>
+          <t>The overlay composer accepts dropped images, OCRs them on-device, and attaches extracted text as pending screen context.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; Command-Option-M</t>
+          <t>Overlay composer drag-and-drop</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Core/Screenshot/OCRService.swift</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2616,37 +2620,37 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>AST-007</t>
+          <t>MOD-001</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Modes</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Listener-mode research actions</t>
+          <t>Mode switching during a session</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>As a passive observer, I want RTI to switch from speaking advice to observation-centric research prompts.</t>
+          <t>As a user, I want to change assistant mode mid-meeting so the next response follows a different system prompt or reference context.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Listener mode exposes Key Tensions, What's Unsaid or Probe, and Emerging Themes actions and adjusts Assist and Follow-ups framing for observer sessions.</t>
+          <t>Modes can be switched from the overlay, live transcript window, or command surfaces, and the next LLM turn uses the active mode without restarting the session.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; command palette; hotkeys</t>
+          <t>Overlay more menu; live transcript window; command palette</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/Settings/ModesTab.swift; RTI/Sources/UI/LiveTranscript/LiveTranscriptView.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2665,37 +2669,37 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>AST-008</t>
+          <t>MOD-002</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Modes</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Primary action remap</t>
+          <t>Mode library editing</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want Command-Return to run the quick action I use most.</t>
+          <t>As a user, I want to create, edit, activate, and delete custom modes.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>The primary action can be remapped to any eligible assistant action, persists in user defaults, and is reflected in the actions menu and command surfaces.</t>
+          <t>Settings list built-in and custom modes, support add and save, block deletion of built-ins, and allow system prompt plus reference text editing.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; menu</t>
+          <t>Settings &gt; Modes</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/LLM/LLMController.swift; RTI/Core/LLM/AssistantAction.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
+          <t>RTI/Sources/Settings/ModesTab.swift; RTI/Sources/Modes/ModeStore.swift</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2714,37 +2718,37 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>AST-009</t>
+          <t>PRM-001</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Prompts</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Smart mode toggle</t>
+          <t>Prompt library editing</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to toggle reasoning-heavy responses when the extra latency is worth it.</t>
+          <t>As a user, I want to edit the shipped prompts that RTI uses for different actions.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Smart mode persists to user defaults and flips the LLM pipeline into smart-mode requests unless a given action already forces smart behavior.</t>
+          <t>Settings organize prompts by group, show edited status and changed-default warnings, allow save, revert, reset-one, reset-all, and preview assembled recap prompts.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Menu; command palette; overlay actions menu indicator</t>
+          <t>Sessions Control &gt; Settings &gt; Prompts</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
+          <t>RTI/Sources/Settings/PromptsTab.swift; RTI/Sources/LLM/PromptStore.swift</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2754,46 +2758,50 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>passed-manual</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Manual smoke pass on 2026-06-30: integrated prompt library, grouped list, editor, and export/reset controls render and are navigable in Sessions Control.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>AST-010</t>
+          <t>PRM-002</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Prompts</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Clear current chat</t>
+          <t>Export shipped default prompts</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to wipe the current chat transcript without touching the live meeting transcript.</t>
+          <t>As a user, I want to export the current shipped prompt defaults for offline comparison or prompt-lab work.</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Clearing chat cancels any in-flight stream, removes in-memory assistant entries immediately, and hides auxiliary floating panels without a confirmation modal.</t>
+          <t>Settings can write a JSON export of shipped defaults to a user-selected location and surface errors with a native alert.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Menu; overlay more menu; command palette</t>
+          <t>Settings &gt; Prompts</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/AppDelegate.swift; RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
+          <t>RTI/Sources/Settings/PromptsTab.swift</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2812,37 +2820,37 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>AST-011</t>
+          <t>GLO-001</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Glossary</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Streaming status and cancellation</t>
+          <t>Glossary editing and parsing</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to see when RTI is still thinking or using a tool and stop it if needed.</t>
+          <t>As a user, I want to maintain a glossary of names and terms so RTI preserves them across LLM outputs.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>While a response streams, the chat tracks streaming and reasoning state plus tool status; the composer swaps send for stop and cancellation prunes empty assistant output.</t>
+          <t>Settings allow multiline glossary editing, ignore comment headers, parse term lines, and show whether parsed entries are currently being sent with every LLM call.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Overlay chat</t>
+          <t>Sessions Control &gt; Settings &gt; Glossary</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
+          <t>RTI/Sources/Settings/GlossaryTab.swift; RTI/Sources/Settings/GlossaryStore.swift</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2852,46 +2860,50 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>passed-manual</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
-      <c r="K48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Manual smoke pass on 2026-06-30: glossary instructions, editable text area, and parsed-entry status surface render correctly in unified control.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>AST-012</t>
+          <t>SET-001</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Assistant provider hot swap</t>
+          <t>Transcription provider selection</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to switch LLM providers without restarting RTI so the next assistant turn uses a different backend immediately.</t>
+          <t>As a user, I want to choose which speech-to-text provider RTI uses.</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Assistant provider selection persists, is exposed in Providers settings plus menu and overlay quick-switch surfaces, and the next LLM request resolves the newly active provider at call time.</t>
+          <t>Setup and Providers settings expose provider selection, persist the active provider, and a live change reconnects the streaming client with a short gap; if AssemblyAI is selected without its key, RTI falls back to Soniox.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; Providers; menu; overlay more menu</t>
+          <t>Overlay &gt; Setup; Settings &gt; Providers; menu</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/LLM/LLMProvider.swift; RTI/Sources/LLM/LLMClient.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
+          <t>RTI/Sources/Settings/KeysTab.swift; RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2907,44 +2919,44 @@
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Overlay More-actions menu shows Assistant provider and Transcription provider submenus on fresh app process 2026-06-30.</t>
+          <t>Manual verification confirmed provider radios in Providers settings and provider submenus in overlay More-actions on 2026-06-30.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>AST-013</t>
+          <t>SET-010</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Quick note insertion mode</t>
+          <t>Unified provider settings</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to flip between normal chat and a quick note insert mode with almost no friction.</t>
+          <t>As a user, I want one settings surface for both provider selection and stored credentials so swapping models is simple.</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>The Assist composer shows a visible `Chat`/`Note` toggle during a live session, keeps focus in the field when toggled, inserts note text inline into the transcript on Enter, and then returns to chat mode automatically for one-off notes.</t>
+          <t>The Providers tab combines assistant-provider selection, STT-provider selection, and stored keys for all supported providers, with provider-specific missing-key guidance and no separate assistant/transcription provider sections in General. The Sessions Control workspace now exposes those settings pages directly in its main left rail instead of treating them as a nested settings-within-settings shell.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Overlay composer</t>
+          <t>Sessions Control &gt; Providers / Modes / Prompts / Glossary / General; Settings command</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Sources/UI/Overlay/OverlayInputState.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
+          <t>RTI/Sources/Settings/SettingsView.swift; RTI/Sources/Settings/KeysTab.swift; RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/UI/SessionsControl/SessionsControlView.swift; RTI/Sources/UI/WindowCoordinator.swift</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2960,44 +2972,44 @@
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>UX change implemented 2026-06-30; manual pass still pending.</t>
+          <t>Unified control navigation implemented 2026-06-30; `WindowCoordinator.openSettings()` now lands on the integrated Providers page in Sessions Control.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>SCR-001</t>
+          <t>SET-011</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Screenshot</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Context capture by hotkey or menu</t>
+          <t>Async transcript-upgrade provider selection</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to attach OCR from the current screen to my next assistant turn.</t>
+          <t>As a user, I want a separate provider choice for future transcript upgrades so I can use a better batch provider than the live one.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Capture Screen runs from command surfaces, uses screenshot plus OCR services, and stores extracted text as pending screen context for the next LLM message rather than sending raw images to the model.</t>
+          <t>Providers settings distinguish `Real-time speech-to-text` from `Transcript upgrade (async)`, persist the async provider separately, and store any async-only credentials such as Aliyun without affecting the live lane.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Command-Shift-H; overlay more menu; command palette</t>
+          <t>Settings &gt; Providers</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/Screenshot/ScreenshotManager.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/Soniox/SonioxClient.swift; RTI/Sources/Settings/KeysTab.swift; RTI/Sources/Settings/KeychainStore.swift; RTI/Sources/Secrets.swift</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3007,46 +3019,50 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>automated-pass</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
-      <c r="K51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Architecture split added on 2026-06-30; current app ships settings/docs, not the Upgrade Transcript job itself.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>SCR-002</t>
+          <t>SET-002</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Screenshot</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Image drag-and-drop OCR</t>
+          <t>Audio input selection</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to drop an image onto the composer to extract text into the next message.</t>
+          <t>As a user, I want to pick the microphone or virtual device RTI should use.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>The overlay composer accepts dropped images, OCRs them on-device, and attaches extracted text as pending screen context.</t>
+          <t>Settings list system default plus available input devices, persist a preferred input UID, and apply it on the next session.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Overlay composer drag-and-drop</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Core/Screenshot/OCRService.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/AudioInputDevice.swift</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3065,37 +3081,37 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>MOD-001</t>
+          <t>SET-003</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Modes</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Mode switching during a session</t>
+          <t>Echo cancellation toggle</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to change assistant mode mid-meeting so the next response follows a different system prompt or reference context.</t>
+          <t>As a user, I want to optionally enable acoustic echo cancellation when I am on speakers.</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Modes can be switched from the overlay, live transcript window, or command surfaces, and the next LLM turn uses the active mode without restarting the session.</t>
+          <t>Settings persist an echo-cancellation preference, explain the current risk of silent microphones on some Macs, and apply the choice on the next session.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Overlay more menu; live transcript window; command palette</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/ModesTab.swift; RTI/Sources/UI/LiveTranscript/LiveTranscriptView.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/AudioCaptureManager.swift</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3114,37 +3130,37 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>MOD-002</t>
+          <t>SET-004</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Modes</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Mode library editing</t>
+          <t>Protect Bluetooth headphone volume</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to create, edit, activate, and delete custom modes.</t>
+          <t>As a user, I want RTI to avoid lowering my Bluetooth headphone volume during capture.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Settings list built-in and custom modes, support add and save, block deletion of built-ins, and allow system prompt plus reference text editing.</t>
+          <t>Settings expose a persisted toggle that keeps Bluetooth headphones at full volume by favoring the built-in mic during recording and restoring the earlier mic on stop.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; Modes</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/ModesTab.swift; RTI/Sources/Modes/ModeStore.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/BluetoothMicGuard.swift</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3163,37 +3179,37 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>PRM-001</t>
+          <t>SET-005</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Prompts</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Prompt library editing</t>
+          <t>Launch at login</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to edit the shipped prompts that RTI uses for different actions.</t>
+          <t>As a user, I want RTI to open automatically when I log into my Mac.</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Settings organize prompts by group, show edited status and changed-default warnings, allow save, revert, reset-one, reset-all, and preview assembled recap prompts.</t>
+          <t>Settings reflect the current launch-at-login state, attempt to change it, and restore the previous toggle plus surface an error if the change fails.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Sessions Control &gt; Settings &gt; Prompts</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/PromptsTab.swift; RTI/Sources/LLM/PromptStore.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Settings/LaunchAtLogin.swift</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3203,50 +3219,46 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>passed-manual</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t>Manual smoke pass on 2026-06-30: integrated prompt library, grouped list, editor, and export/reset controls render and are navigable in Sessions Control.</t>
-        </is>
-      </c>
+      <c r="K55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>PRM-002</t>
+          <t>SET-006</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Prompts</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Export shipped default prompts</t>
+          <t>Audio monitor</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to export the current shipped prompt defaults for offline comparison or prompt-lab work.</t>
+          <t>As a user, I want to verify that RTI is capturing both my side and the other party before or during a meeting.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Settings can write a JSON export of shipped defaults to a user-selected location and surface errors with a native alert.</t>
+          <t>Settings embed a live audio monitor with current device and level information; the same monitor is also available from the menubar.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; Prompts</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/PromptsTab.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/UI/AudioMonitor/AudioMonitorView.swift</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3265,37 +3277,37 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>GLO-001</t>
+          <t>SET-007</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Glossary</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Glossary editing and parsing</t>
+          <t>Hotkey reference</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to maintain a glossary of names and terms so RTI preserves them across LLM outputs.</t>
+          <t>As a user, I want a single place to confirm RTI's global shortcuts.</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Settings allow multiline glossary editing, ignore comment headers, parse term lines, and show whether parsed entries are currently being sent with every LLM call.</t>
+          <t>Settings list the principal global hotkeys and explain that Command-Return is remappable while additional quick AI actions live in the command palette.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Sessions Control &gt; Settings &gt; Glossary</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GlossaryTab.swift; RTI/Sources/Settings/GlossaryStore.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3305,20 +3317,16 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>passed-manual</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>Manual smoke pass on 2026-06-30: glossary instructions, editable text area, and parsed-entry status surface render correctly in unified control.</t>
-        </is>
-      </c>
+      <c r="K57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>SET-001</t>
+          <t>SET-008</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3328,27 +3336,27 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Transcription provider selection</t>
+          <t>Data and support actions</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to choose which speech-to-text provider RTI uses.</t>
+          <t>As a user, I want quick access to RTI's support folder, crash log, and logs.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Setup and Providers settings expose provider selection, persist the active provider, and a live change reconnects the streaming client with a short gap; if AssemblyAI is selected without its key, RTI falls back to Soniox.</t>
+          <t>Settings can reveal the RTI Application Support folder, reveal a crash log if one exists, and route to the logs viewer.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Setup; Settings &gt; Providers; menu</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/KeysTab.swift; RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3358,20 +3366,16 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>passed-manual</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
-      <c r="K58" s="2" t="inlineStr">
-        <is>
-          <t>Manual verification confirmed provider radios in Providers settings and provider submenus in overlay More-actions on 2026-06-30.</t>
-        </is>
-      </c>
+      <c r="K58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>SET-010</t>
+          <t>SET-009</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3381,27 +3385,27 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Unified provider settings</t>
+          <t>Diagnostics copy</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want one settings surface for both provider selection and stored credentials so swapping models is simple.</t>
+          <t>As a user, I want to copy a concise diagnostics bundle for support or debugging.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>The Providers tab combines assistant-provider selection, STT-provider selection, and stored keys for all supported providers, with provider-specific missing-key guidance and no separate assistant/transcription provider sections in General. The Sessions Control workspace now exposes those settings pages directly in its main left rail instead of treating them as a nested settings-within-settings shell.</t>
+          <t>Settings surface version, model, and provider diagnostics and can copy a formatted diagnostics block to the pasteboard.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Sessions Control &gt; Providers / Modes / Prompts / Glossary / General; Settings command</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/SettingsView.swift; RTI/Sources/Settings/KeysTab.swift; RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/UI/SessionsControl/SessionsControlView.swift; RTI/Sources/UI/WindowCoordinator.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3411,50 +3415,46 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>automated-pass</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
-      <c r="K59" s="2" t="inlineStr">
-        <is>
-          <t>Unified control navigation implemented 2026-06-30; `WindowCoordinator.openSettings()` now lands on the integrated Providers page in Sessions Control.</t>
-        </is>
-      </c>
+      <c r="K59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>SET-011</t>
+          <t>DOC-001</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Async transcript-upgrade provider selection</t>
+          <t>Transcription lane documentation</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want a separate provider choice for future transcript upgrades so I can use a better batch provider than the live one.</t>
+          <t>As a developer or operator, I want clear documentation for live transcription versus future transcript upgrades so provider choices are unambiguous.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Providers settings distinguish `Real-time speech-to-text` from `Transcript upgrade (async)`, persist the async provider separately, and store any async-only credentials such as Aliyun without affecting the live lane.</t>
+          <t>Docs explain that real-time STT and async transcript upgrade are separate lanes, recommend provider defaults per laneand describe how the Upgrade Transcript action replaces the rough transcript.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; Providers</t>
+          <t>README; docs</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Soniox/SonioxClient.swift; RTI/Sources/Settings/KeysTab.swift; RTI/Sources/Settings/KeychainStore.swift; RTI/Sources/Secrets.swift</t>
+          <t>README.md; docs/transcript-upgrade-providers.md</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3470,44 +3470,44 @@
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Architecture split added on 2026-06-30; current app ships settings/docs, not the Upgrade Transcript job itself.</t>
+          <t>Documentation added 2026-06-30 and tied to the transcribe skill’s provider defaults.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>SET-002</t>
+          <t>LOG-001</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Logs</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Audio input selection</t>
+          <t>Live and past logs viewer</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to pick the microphone or virtual device RTI should use.</t>
+          <t>As a user, I want to inspect RTI's current and past application logs without opening files manually.</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Settings list system default plus available input devices, persist a preferred input UID, and apply it on the next session.</t>
+          <t>The logs window switches between live in-memory entries and past daily files, supports copy, clear or reveal actions appropriate to each mode, and shows the crash log in an expandable section.</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; General</t>
+          <t>Sessions Control &gt; Logs</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/AudioInputDevice.swift</t>
+          <t>RTI/Sources/Settings/LogsView.swift; RTI/Sources/Support/AppLog.swift; RTI/Sources/Support/CrashLog.swift</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3517,46 +3517,50 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>passed-manual</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Manual smoke pass on 2026-06-30: verified live/past toggle, past-date selector, copy/reveal controls, and crash-log disclosure inside Sessions Control.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>SET-003</t>
+          <t>ARC-001</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Archive</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Echo cancellation toggle</t>
+          <t>Session archive browser</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to optionally enable acoustic echo cancellation when I am on speakers.</t>
+          <t>As a user, I want to read past RTI sessions inside the app after they are saved.</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Settings persist an echo-cancellation preference, explain the current risk of silent microphones on some Macs, and apply the choice on the next session.</t>
+          <t>The Sessions browser loads recent archive folders, groups them by date buckets, opens a selected session, and defaults to the highest-priority available file.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; General</t>
+          <t>Sessions window &gt; Sessions; notifications; overlay more menu</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/AudioCaptureManager.swift</t>
+          <t>RTI/Sources/UI/SessionsControl/SessionsBrowserView.swift; RTI/Sources/Session/SessionArchive.swift; RTI/Sources/UI/WindowCoordinator.swift</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3575,37 +3579,37 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>SET-004</t>
+          <t>ARC-002</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Archive</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Protect Bluetooth headphone volume</t>
+          <t>Session file copy and export</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to avoid lowering my Bluetooth headphone volume during capture.</t>
+          <t>As a user, I want to copy or export archived session files for sharing or further work outside RTI.</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Settings expose a persisted toggle that keeps Bluetooth headphones at full volume by favoring the built-in mic during recording and restoring the earlier mic on stop.</t>
+          <t>The Sessions browser can copy the current markdown, export markdown, export PDF, and reveal the backing session folder in Finder.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; General</t>
+          <t>Sessions window &gt; Sessions</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/BluetoothMicGuard.swift</t>
+          <t>RTI/Sources/UI/SessionsControl/SessionsBrowserView.swift</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3624,37 +3628,37 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>SET-005</t>
+          <t>ARC-003</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Archive</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Launch at login</t>
+          <t>End-of-session writeout</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to open automatically when I log into my Mac.</t>
+          <t>As a user, I want RTI to preserve text artifacts from a finished session without keeping audio.</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Settings reflect the current launch-at-login state, attempt to change it, and restore the previous toggle plus surface an error if the change fails.</t>
+          <t>On stop, RTI can write transcript, chat, and screen-context artifacts into a timestamped session folder with owner-only permissions; live translation tokens are excluded from the kept transcript.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; General</t>
+          <t>Implicit session lifecycle</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Settings/LaunchAtLogin.swift</t>
+          <t>RTI/Sources/Session/SessionArchive.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3673,37 +3677,37 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>SET-006</t>
+          <t>ARC-005</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Archive</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Audio monitor</t>
+          <t>Session-local retained audio</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to verify that RTI is capturing both my side and the other party before or during a meeting.</t>
+          <t>As a user, I want any retained session audio to live beside the transcript so the session folder is self-contained for upgrades and review.</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Settings embed a live audio monitor with current device and level information; the same monitor is also available from the menubar.</t>
+          <t>When a session is archived, any kept `mic` and `system` `.m4a` files are moved into that session folder as `audio-mic.m4a` and `audio-system.m4a` on a best-effort basis.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; General</t>
+          <t>Implicit session lifecycle</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/UI/AudioMonitor/AudioMonitorView.swift</t>
+          <t>RTI/Sources/Session/SessionArchive.swift; RTI/Sources/Session/SessionCoordinator.swift; RTI/Sources/Audio/WAVWriter.swift</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3713,509 +3717,11 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>automated-pass</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
-      <c r="K65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>SET-007</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Hotkey reference</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>As a user, I want a single place to confirm RTI's global shortcuts.</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Settings list the principal global hotkeys and explain that Command-Return is remappable while additional quick AI actions live in the command palette.</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>Settings &gt; General</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>not-tested</t>
-        </is>
-      </c>
-      <c r="J66" s="2" t="inlineStr"/>
-      <c r="K66" s="2" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>SET-008</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Data and support actions</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>As a user, I want quick access to RTI's support folder, crash log, and logs.</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Settings can reveal the RTI Application Support folder, reveal a crash log if one exists, and route to the logs viewer.</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>Settings &gt; General</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>not-tested</t>
-        </is>
-      </c>
-      <c r="J67" s="2" t="inlineStr"/>
-      <c r="K67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>SET-009</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Diagnostics copy</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>As a user, I want to copy a concise diagnostics bundle for support or debugging.</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Settings surface version, model, and provider diagnostics and can copy a formatted diagnostics block to the pasteboard.</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>Settings &gt; General</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>not-tested</t>
-        </is>
-      </c>
-      <c r="J68" s="2" t="inlineStr"/>
-      <c r="K68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>DOC-001</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>Transcription lane documentation</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>As a developer or operator, I want clear documentation for live transcription versus future transcript upgrades so provider choices and summary regeneration behavior are unambiguous.</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>Docs explain that real-time STT and async transcript upgrade are separate lanes, recommend provider defaults per lane, and describe how a future Upgrade Transcript action should regenerate the summary from upgraded text.</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>README; docs</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>README.md; docs/transcript-upgrade-providers.md</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>automated-pass</t>
-        </is>
-      </c>
-      <c r="J69" s="2" t="inlineStr"/>
-      <c r="K69" s="2" t="inlineStr">
-        <is>
-          <t>Documentation added 2026-06-30 and tied to the transcribe skill’s provider defaults.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>LOG-001</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Logs</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Live and past logs viewer</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>As a user, I want to inspect RTI's current and past application logs without opening files manually.</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>The logs window switches between live in-memory entries and past daily files, supports copy, clear or reveal actions appropriate to each mode, and shows the crash log in an expandable section.</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>Sessions Control &gt; Logs</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>RTI/Sources/Settings/LogsView.swift; RTI/Sources/Support/AppLog.swift; RTI/Sources/Support/CrashLog.swift</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>passed-manual</t>
-        </is>
-      </c>
-      <c r="J70" s="2" t="inlineStr"/>
-      <c r="K70" s="2" t="inlineStr">
-        <is>
-          <t>Manual smoke pass on 2026-06-30: verified live/past toggle, past-date selector, copy/reveal controls, and crash-log disclosure inside Sessions Control.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>ARC-001</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>Archive</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>Session archive browser</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>As a user, I want to read past RTI sessions inside the app after they are saved.</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>The Sessions browser loads recent archive folders, groups them by date buckets, opens a selected session, and defaults to the highest-priority available file.</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>Sessions window &gt; Sessions; notifications; overlay more menu</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="inlineStr">
-        <is>
-          <t>RTI/Sources/UI/SessionsControl/SessionsBrowserView.swift; RTI/Sources/Session/SessionArchive.swift; RTI/Sources/UI/WindowCoordinator.swift</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>not-tested</t>
-        </is>
-      </c>
-      <c r="J71" s="2" t="inlineStr"/>
-      <c r="K71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>ARC-002</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>Archive</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>Session file copy and export</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>As a user, I want to copy or export archived session files for sharing or further work outside RTI.</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>The Sessions browser can copy the current markdown, export markdown, export PDF, and reveal the backing session folder in Finder.</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>Sessions window &gt; Sessions</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>RTI/Sources/UI/SessionsControl/SessionsBrowserView.swift</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>not-tested</t>
-        </is>
-      </c>
-      <c r="J72" s="2" t="inlineStr"/>
-      <c r="K72" s="2" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>ARC-003</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>Archive</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>End-of-session writeout</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>As a user, I want RTI to preserve text artifacts from a finished session without keeping audio.</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>On stop, RTI can write transcript, chat, notes, discussion-guide, findings, and summary artifacts into a timestamped session folder with owner-only permissions; live translation tokens are excluded from the kept transcript.</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>Implicit session lifecycle</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr">
-        <is>
-          <t>RTI/Sources/Session/SessionArchive.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
-        </is>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>not-tested</t>
-        </is>
-      </c>
-      <c r="J73" s="2" t="inlineStr"/>
-      <c r="K73" s="2" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>ARC-004</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>Archive</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Summary-ready notification deep link</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>As a user, I want a notification when the post-stop summary is ready and a direct path into that session.</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>When auto-summary finishes, RTI posts a local notification carrying the session folder; clicking it activates RTI and opens that exact session in the browser.</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>Post-stop notification</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>RTI/Sources/Session/SessionArchive.swift; RTI/Sources/AppDelegate.swift; RTI/Sources/UI/WindowCoordinator.swift</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>not-tested</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr"/>
-      <c r="K74" s="2" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>ARC-005</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>Archive</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>Session-local retained audio</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>As a user, I want any retained session audio to live beside the transcript and summary so the session folder is self-contained for upgrades and review.</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>When a session is archived, any kept `mic` and `system` `.m4a` files are moved into that session folder as `audio-mic.m4a` and `audio-system.m4a` on a best-effort basis.</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>Implicit session lifecycle</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>RTI/Sources/Session/SessionArchive.swift; RTI/Sources/Session/SessionCoordinator.swift; RTI/Sources/Audio/WAVWriter.swift</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t>automated-pass</t>
-        </is>
-      </c>
-      <c r="J75" s="2" t="inlineStr"/>
-      <c r="K75" s="2" t="inlineStr">
+      <c r="K65" s="2" t="inlineStr">
         <is>
           <t>Forward path implemented 2026-06-30; retroactive migration for old recordings remains to be done conservatively.</t>
         </is>
@@ -4249,6 +3755,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -4268,7 +3775,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
@@ -4291,7 +3798,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Prompts, Glossary, Logs, Setup nav, provider/settings integration, and Findings toggle have manual evidence</t>
+          <t>Prompts, Glossary, Logs, Setup nav, and provider/settings integration have manual evidence</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore live Notes after the analysis trim
Notes is the one in-app analysis feature Tristan wants kept. It comes back as it
was before 7927d17d: the Notes tab (cmd-5, on by default), the periodic
NotesGenerationController, the Live notes prompt, the Settings toggle and
interval under the same stored keys, notes.md in the session archive, and a
Generated notes section in the -rti.md sidecar. The Sessions window lists Notes
first again.

Notes now run on AutoAssistScheduler and read the transcript through
TranscriptContext, so neither the old AnalysisScheduler nor TranscriptAnalysis
returns. Summaries, generated titles, the discussion guide and Findings stay
removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VydPNw8QreBBTMDGVc2fsn
</commit_message>
<xml_diff>
--- a/docs/rti_feature_tracker.xlsx
+++ b/docs/rti_feature_tracker.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1828,7 +1828,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ANA-005</t>
+          <t>ANA-001</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1838,27 +1838,27 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Enable Auto live analysis</t>
+          <t>Enable Notes live analysis</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to proactively surface suggestions only when I opt into that behavior.</t>
+          <t>As a user, I want to turn Notes off when I do not need it so the extra live analysis stays optional.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Auto is opt-in, appears as a live panel toggle, and when enabled schedules proactive card generation plus quiet-window debounced generation after speech settles.</t>
+          <t>Notes is on by default, appears as a live panel toggle in Prepare and Settings &gt; General with an interval slider, and when enabled adds the Notes tab and lets the scheduler generate note batches during the session.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Setup</t>
+          <t>Overlay &gt; Setup; Settings &gt; General</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Session/SessionCoordinator.swift; RTI/Sources/Analysis/AutoAssistController.swift</t>
+          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1871,13 +1871,13 @@
           <t>not-tested</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ANA-006</t>
+          <t>ANA-002</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1887,27 +1887,27 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Auto tab suggestions</t>
+          <t>Notes tab controls</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want live proactive suggestions about what to say, ask, recall, or flag.</t>
+          <t>As a user, I want to manually regenerate, copy, and export generated notes.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>The Auto tab shows SAY, ASK, RECALL, and FLAG cards, manual resurface, copy support, and unseen-count semantics when the user has not viewed the tab.</t>
+          <t>The Notes tab shows progress, errors, note blocks with time ranges, copy-per-block, copy-all, regenerate-now, and export-to-markdown actions. At stop the blocks are written to notes.md and the -rti.md sidecar.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Auto</t>
+          <t>Overlay &gt; Notes</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Analysis/AutoAssistController.swift</t>
+          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Notes/NotesGenerationController.swift; RTI/Sources/Session/SessionArchive.swift</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1920,43 +1920,43 @@
           <t>not-tested</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>AST-001</t>
+          <t>ANA-005</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Freeform ask-anything composer</t>
+          <t>Enable Auto live analysis</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to type my own question to RTI instead of relying only on canned actions.</t>
+          <t>As a user, I want RTI to proactively surface suggestions only when I opt into that behavior.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>The overlay composer accepts freeform text, submits on Return, clears draft on session stop, and routes the text through the standard LLM pipeline.</t>
+          <t>Auto is opt-in, appears as a live panel toggle, and when enabled schedules proactive card generation plus quiet-window debounced generation after speech settles.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Overlay composer</t>
+          <t>Overlay &gt; Setup</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Session/SessionCoordinator.swift; RTI/Sources/Analysis/AutoAssistController.swift</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -1975,37 +1975,37 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>AST-002</t>
+          <t>ANA-006</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Assistant</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Assist quick action</t>
+          <t>Auto tab suggestions</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to suggest what I should say next.</t>
+          <t>As a user, I want live proactive suggestions about what to say, ask, recall, or flag.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>The Assist action sends the current prompt-store Assist prompt, grounded in recent transcript and meeting context, and streams a response into the chat.</t>
+          <t>The Auto tab shows SAY, ASK, RECALL, and FLAG cards, manual resurface, copy support, and unseen-count semantics when the user has not viewed the tab.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; Command-Return; command palette</t>
+          <t>Overlay &gt; Auto</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/Analysis/AutoAssistController.swift</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2024,7 +2024,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>AST-003</t>
+          <t>AST-001</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2034,27 +2034,27 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Say Next quick action</t>
+          <t>Freeform ask-anything composer</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want a terse one-line draft reply.</t>
+          <t>As a user, I want to type my own question to RTI instead of relying only on canned actions.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>The Say Next action is available as a quick action and global hotkey and requests a one-line reply through the assistant pipeline.</t>
+          <t>The overlay composer accepts freeform text, submits on Return, clears draft on session stop, and routes the text through the standard LLM pipeline.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; Command-Option-S</t>
+          <t>Overlay composer</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2073,7 +2073,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>AST-004</t>
+          <t>AST-002</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2083,22 +2083,22 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Follow-up Questions quick action</t>
+          <t>Assist quick action</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to propose follow-up questions based on the conversation.</t>
+          <t>As a user, I want RTI to suggest what I should say next.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>The Follow-ups action uses its prompt-store prompt, and streams results in chat.</t>
+          <t>The Assist action sends the current prompt-store Assist prompt, grounded in recent transcript and meeting context, and streams a response into the chat.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; Command-Option-F</t>
+          <t>Overlay actions menu; Command-Return; command palette</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2122,7 +2122,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>AST-005</t>
+          <t>AST-003</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2132,27 +2132,27 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Recap quick action and recap depth</t>
+          <t>Say Next quick action</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want fast recaps at different levels of detail.</t>
+          <t>As a user, I want a terse one-line draft reply.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>RTI offers Recap as an action, persists a sticky recap depth, and also supports brief and detailed one-shot recap variants via commands.</t>
+          <t>The Say Next action is available as a quick action and global hotkey and requests a one-line reply through the assistant pipeline.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; Command-Option-R; command palette</t>
+          <t>Overlay actions menu; Command-Option-S</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
+          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2171,7 +2171,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>AST-007</t>
+          <t>AST-004</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2181,22 +2181,22 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Listener-mode research actions</t>
+          <t>Follow-up Questions quick action</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>As a passive observer, I want RTI to switch from speaking advice to observation-centric research prompts.</t>
+          <t>As a user, I want RTI to propose follow-up questions based on the conversation.</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Listener mode exposes Key Tensions, What's Unsaid or Probe, and Emerging Themes actions and adjusts Assist and Follow-ups framing for observer sessions.</t>
+          <t>The Follow-ups action uses its prompt-store prompt, and streams results in chat.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; command palette; hotkeys</t>
+          <t>Overlay actions menu; Command-Option-F</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2220,7 +2220,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>AST-008</t>
+          <t>AST-005</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2230,27 +2230,27 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Primary action remap</t>
+          <t>Recap quick action and recap depth</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want Command-Return to run the quick action I use most.</t>
+          <t>As a user, I want fast recaps at different levels of detail.</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>The primary action can be remapped to any eligible assistant action, persists in user defaults, and is reflected in the actions menu and command surfaces.</t>
+          <t>RTI offers Recap as an action, persists a sticky recap depth, and also supports brief and detailed one-shot recap variants via commands.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Overlay actions menu; menu</t>
+          <t>Overlay actions menu; Command-Option-R; command palette</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/LLM/LLMController.swift; RTI/Core/LLM/AssistantAction.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
+          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2269,7 +2269,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>AST-009</t>
+          <t>AST-007</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2279,27 +2279,27 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Smart mode toggle</t>
+          <t>Listener-mode research actions</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to toggle reasoning-heavy responses when the extra latency is worth it.</t>
+          <t>As a passive observer, I want RTI to switch from speaking advice to observation-centric research prompts.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Smart mode persists to user defaults and flips the LLM pipeline into smart-mode requests unless a given action already forces smart behavior.</t>
+          <t>Listener mode exposes Key Tensions, What's Unsaid or Probe, and Emerging Themes actions and adjusts Assist and Follow-ups framing for observer sessions.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Menu; command palette; overlay actions menu indicator</t>
+          <t>Overlay actions menu; command palette; hotkeys</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
+          <t>RTI/Core/LLM/AssistantAction.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2318,7 +2318,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AST-010</t>
+          <t>AST-008</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2328,27 +2328,27 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Clear current chat</t>
+          <t>Primary action remap</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to wipe the current chat transcript without touching the live meeting transcript.</t>
+          <t>As a user, I want Command-Return to run the quick action I use most.</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Clearing chat cancels any in-flight stream, removes in-memory assistant entries immediately, and hides auxiliary floating panels without a confirmation modal.</t>
+          <t>The primary action can be remapped to any eligible assistant action, persists in user defaults, and is reflected in the actions menu and command surfaces.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Menu; overlay more menu; command palette</t>
+          <t>Overlay actions menu; menu</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/AppDelegate.swift; RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
+          <t>RTI/Sources/LLM/LLMController.swift; RTI/Core/LLM/AssistantAction.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2367,7 +2367,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AST-011</t>
+          <t>AST-009</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2377,27 +2377,27 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Streaming status and cancellation</t>
+          <t>Smart mode toggle</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to see when RTI is still thinking or using a tool and stop it if needed.</t>
+          <t>As a user, I want to toggle reasoning-heavy responses when the extra latency is worth it.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>While a response streams, the chat tracks streaming and reasoning state plus tool status; the composer swaps send for stop and cancellation prunes empty assistant output.</t>
+          <t>Smart mode persists to user defaults and flips the LLM pipeline into smart-mode requests unless a given action already forces smart behavior.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Overlay chat</t>
+          <t>Menu; command palette; overlay actions menu indicator</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
+          <t>RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2416,7 +2416,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AST-012</t>
+          <t>AST-010</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2426,27 +2426,27 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Assistant provider hot swap</t>
+          <t>Clear current chat</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to switch LLM providers without restarting RTI so the next assistant turn uses a different backend immediately.</t>
+          <t>As a user, I want to wipe the current chat transcript without touching the live meeting transcript.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Assistant provider selection persists, is exposed in Providers settings plus menu and overlay quick-switch surfaces, and the next LLM request resolves the newly active provider at call time.</t>
+          <t>Clearing chat cancels any in-flight stream, removes in-memory assistant entries immediately, and hides auxiliary floating panels without a confirmation modal.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; Providers; menu; overlay more menu</t>
+          <t>Menu; overlay more menu; command palette</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/LLM/LLMProvider.swift; RTI/Sources/LLM/LLMClient.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
+          <t>RTI/Sources/AppDelegate.swift; RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2456,20 +2456,16 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>passed-manual</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>Overlay More-actions menu shows Assistant provider and Transcription provider submenus on fresh app process 2026-06-30.</t>
-        </is>
-      </c>
+      <c r="K40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>AST-013</t>
+          <t>AST-011</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2479,27 +2475,27 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Quick note insertion mode</t>
+          <t>Streaming status and cancellation</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to flip between normal chat and a quick note insert mode with almost no friction.</t>
+          <t>As a user, I want to see when RTI is still thinking or using a tool and stop it if needed.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>The Assist composer shows a visible `Chat`/`Note` toggle during a live session, keeps focus in the field when toggled, inserts note text inline into the transcript on Enter, and then returns to chat mode automatically for one-off notes.</t>
+          <t>While a response streams, the chat tracks streaming and reasoning state plus tool status; the composer swaps send for stop and cancellation prunes empty assistant output.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Overlay composer</t>
+          <t>Overlay chat</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Sources/UI/Overlay/OverlayInputState.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
+          <t>RTI/Sources/LLM/LLMController.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2509,50 +2505,46 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>automated-pass</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>UX change implemented 2026-06-30; manual pass still pending.</t>
-        </is>
-      </c>
+      <c r="K41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>SCR-001</t>
+          <t>AST-012</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Screenshot</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Context capture by hotkey or menu</t>
+          <t>Assistant provider hot swap</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to attach OCR from the current screen to my next assistant turn.</t>
+          <t>As a user, I want to switch LLM providers without restarting RTI so the next assistant turn uses a different backend immediately.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Capture Screen runs from command surfaces, uses screenshot plus OCR services, and stores extracted text as pending screen context for the next LLM message rather than sending raw images to the model.</t>
+          <t>Assistant provider selection persists, is exposed in Providers settings plus menu and overlay quick-switch surfaces, and the next LLM request resolves the newly active provider at call time.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Command-Shift-H; overlay more menu; command palette</t>
+          <t>Settings &gt; Providers; menu; overlay more menu</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/Screenshot/ScreenshotManager.swift; RTI/Sources/LLM/LLMController.swift</t>
+          <t>RTI/Sources/LLM/LLMProvider.swift; RTI/Sources/LLM/LLMClient.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2562,46 +2554,50 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>passed-manual</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Overlay More-actions menu shows Assistant provider and Transcription provider submenus on fresh app process 2026-06-30.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>SCR-002</t>
+          <t>AST-013</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Screenshot</t>
+          <t>Assistant</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Image drag-and-drop OCR</t>
+          <t>Quick note insertion mode</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to drop an image onto the composer to extract text into the next message.</t>
+          <t>As a user, I want to flip between normal chat and a quick note insert mode with almost no friction.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>The overlay composer accepts dropped images, OCRs them on-device, and attaches extracted text as pending screen context.</t>
+          <t>The Assist composer shows a visible `Chat`/`Note` toggle during a live session, keeps focus in the field when toggled, inserts note text inline into the transcript on Enter, and then returns to chat mode automatically for one-off notes.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Overlay composer drag-and-drop</t>
+          <t>Overlay composer</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Core/Screenshot/OCRService.swift</t>
+          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Sources/UI/Overlay/OverlayInputState.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2611,46 +2607,50 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>automated-pass</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>UX change implemented 2026-06-30; manual pass still pending.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>MOD-001</t>
+          <t>SCR-001</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Modes</t>
+          <t>Screenshot</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Mode switching during a session</t>
+          <t>Context capture by hotkey or menu</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to change assistant mode mid-meeting so the next response follows a different system prompt or reference context.</t>
+          <t>As a user, I want to attach OCR from the current screen to my next assistant turn.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Modes can be switched from the overlay, live transcript window, or command surfaces, and the next LLM turn uses the active mode without restarting the session.</t>
+          <t>Capture Screen runs from command surfaces, uses screenshot plus OCR services, and stores extracted text as pending screen context for the next LLM message rather than sending raw images to the model.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Overlay more menu; live transcript window; command palette</t>
+          <t>Command-Shift-H; overlay more menu; command palette</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/ModesTab.swift; RTI/Sources/UI/LiveTranscript/LiveTranscriptView.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
+          <t>RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/Screenshot/ScreenshotManager.swift; RTI/Sources/LLM/LLMController.swift</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -2669,37 +2669,37 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>MOD-002</t>
+          <t>SCR-002</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Modes</t>
+          <t>Screenshot</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Mode library editing</t>
+          <t>Image drag-and-drop OCR</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to create, edit, activate, and delete custom modes.</t>
+          <t>As a user, I want to drop an image onto the composer to extract text into the next message.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Settings list built-in and custom modes, support add and save, block deletion of built-ins, and allow system prompt plus reference text editing.</t>
+          <t>The overlay composer accepts dropped images, OCRs them on-device, and attaches extracted text as pending screen context.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; Modes</t>
+          <t>Overlay composer drag-and-drop</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/ModesTab.swift; RTI/Sources/Modes/ModeStore.swift</t>
+          <t>RTI/Sources/UI/Overlay/AssistantInputView.swift; RTI/Core/Screenshot/OCRService.swift</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2718,37 +2718,37 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>PRM-001</t>
+          <t>MOD-001</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Prompts</t>
+          <t>Modes</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Prompt library editing</t>
+          <t>Mode switching during a session</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to edit the shipped prompts that RTI uses for different actions.</t>
+          <t>As a user, I want to change assistant mode mid-meeting so the next response follows a different system prompt or reference context.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Settings organize prompts by group, show edited status and changed-default warnings, allow save, revert, reset-one, reset-all, and preview assembled recap prompts.</t>
+          <t>Modes can be switched from the overlay, live transcript window, or command surfaces, and the next LLM turn uses the active mode without restarting the session.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Sessions Control &gt; Settings &gt; Prompts</t>
+          <t>Overlay more menu; live transcript window; command palette</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/PromptsTab.swift; RTI/Sources/LLM/PromptStore.swift</t>
+          <t>RTI/Sources/Settings/ModesTab.swift; RTI/Sources/UI/LiveTranscript/LiveTranscriptView.swift; RTI/Sources/UI/Overlay/AssistantInputView.swift</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2758,50 +2758,46 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>passed-manual</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>Manual smoke pass on 2026-06-30: integrated prompt library, grouped list, editor, and export/reset controls render and are navigable in Sessions Control.</t>
-        </is>
-      </c>
+      <c r="K46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>PRM-002</t>
+          <t>MOD-002</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Prompts</t>
+          <t>Modes</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Export shipped default prompts</t>
+          <t>Mode library editing</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to export the current shipped prompt defaults for offline comparison or prompt-lab work.</t>
+          <t>As a user, I want to create, edit, activate, and delete custom modes.</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Settings can write a JSON export of shipped defaults to a user-selected location and surface errors with a native alert.</t>
+          <t>Settings list built-in and custom modes, support add and save, block deletion of built-ins, and allow system prompt plus reference text editing.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; Prompts</t>
+          <t>Settings &gt; Modes</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/PromptsTab.swift</t>
+          <t>RTI/Sources/Settings/ModesTab.swift; RTI/Sources/Modes/ModeStore.swift</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -2820,37 +2816,37 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GLO-001</t>
+          <t>PRM-001</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Glossary</t>
+          <t>Prompts</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Glossary editing and parsing</t>
+          <t>Prompt library editing</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to maintain a glossary of names and terms so RTI preserves them across LLM outputs.</t>
+          <t>As a user, I want to edit the shipped prompts that RTI uses for different actions.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Settings allow multiline glossary editing, ignore comment headers, parse term lines, and show whether parsed entries are currently being sent with every LLM call.</t>
+          <t>Settings organize prompts by group, show edited status and changed-default warnings, allow save, revert, reset-one, reset-all, and preview assembled recap prompts.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Sessions Control &gt; Settings &gt; Glossary</t>
+          <t>Sessions Control &gt; Settings &gt; Prompts</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GlossaryTab.swift; RTI/Sources/Settings/GlossaryStore.swift</t>
+          <t>RTI/Sources/Settings/PromptsTab.swift; RTI/Sources/LLM/PromptStore.swift</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2866,44 +2862,44 @@
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Manual smoke pass on 2026-06-30: glossary instructions, editable text area, and parsed-entry status surface render correctly in unified control.</t>
+          <t>Manual smoke pass on 2026-06-30: integrated prompt library, grouped list, editor, and export/reset controls render and are navigable in Sessions Control.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>SET-001</t>
+          <t>PRM-002</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Prompts</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Transcription provider selection</t>
+          <t>Export shipped default prompts</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to choose which speech-to-text provider RTI uses.</t>
+          <t>As a user, I want to export the current shipped prompt defaults for offline comparison or prompt-lab work.</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Setup and Providers settings expose provider selection, persist the active provider, and a live change reconnects the streaming client with a short gap; if AssemblyAI is selected without its key, RTI falls back to Soniox.</t>
+          <t>Settings can write a JSON export of shipped defaults to a user-selected location and surface errors with a native alert.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Overlay &gt; Setup; Settings &gt; Providers; menu</t>
+          <t>Settings &gt; Prompts</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/KeysTab.swift; RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
+          <t>RTI/Sources/Settings/PromptsTab.swift</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2913,50 +2909,46 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>passed-manual</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
-      <c r="K49" s="2" t="inlineStr">
-        <is>
-          <t>Manual verification confirmed provider radios in Providers settings and provider submenus in overlay More-actions on 2026-06-30.</t>
-        </is>
-      </c>
+      <c r="K49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>SET-010</t>
+          <t>GLO-001</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Settings</t>
+          <t>Glossary</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Unified provider settings</t>
+          <t>Glossary editing and parsing</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want one settings surface for both provider selection and stored credentials so swapping models is simple.</t>
+          <t>As a user, I want to maintain a glossary of names and terms so RTI preserves them across LLM outputs.</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>The Providers tab combines assistant-provider selection, STT-provider selection, and stored keys for all supported providers, with provider-specific missing-key guidance and no separate assistant/transcription provider sections in General. The Sessions Control workspace now exposes those settings pages directly in its main left rail instead of treating them as a nested settings-within-settings shell.</t>
+          <t>Settings allow multiline glossary editing, ignore comment headers, parse term lines, and show whether parsed entries are currently being sent with every LLM call.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Sessions Control &gt; Providers / Modes / Prompts / Glossary / General; Settings command</t>
+          <t>Sessions Control &gt; Settings &gt; Glossary</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/SettingsView.swift; RTI/Sources/Settings/KeysTab.swift; RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/UI/SessionsControl/SessionsControlView.swift; RTI/Sources/UI/WindowCoordinator.swift</t>
+          <t>RTI/Sources/Settings/GlossaryTab.swift; RTI/Sources/Settings/GlossaryStore.swift</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2966,20 +2958,20 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>automated-pass</t>
+          <t>passed-manual</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Unified control navigation implemented 2026-06-30; `WindowCoordinator.openSettings()` now lands on the integrated Providers page in Sessions Control.</t>
+          <t>Manual smoke pass on 2026-06-30: glossary instructions, editable text area, and parsed-entry status surface render correctly in unified control.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>SET-011</t>
+          <t>SET-001</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2989,27 +2981,27 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Async transcript-upgrade provider selection</t>
+          <t>Transcription provider selection</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want a separate provider choice for future transcript upgrades so I can use a better batch provider than the live one.</t>
+          <t>As a user, I want to choose which speech-to-text provider RTI uses.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Providers settings distinguish `Real-time speech-to-text` from `Transcript upgrade (async)`, persist the async provider separately, and store any async-only credentials such as Aliyun without affecting the live lane.</t>
+          <t>Setup and Providers settings expose provider selection, persist the active provider, and a live change reconnects the streaming client with a short gap; if AssemblyAI is selected without its key, RTI falls back to Soniox.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; Providers</t>
+          <t>Overlay &gt; Setup; Settings &gt; Providers; menu</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Soniox/SonioxClient.swift; RTI/Sources/Settings/KeysTab.swift; RTI/Sources/Settings/KeychainStore.swift; RTI/Sources/Secrets.swift</t>
+          <t>RTI/Sources/Settings/KeysTab.swift; RTI/Sources/UI/Overlay/OverlayTabs.swift; RTI/Sources/UI/CommandPalette/CommandPaletteFactory.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3019,20 +3011,20 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>automated-pass</t>
+          <t>passed-manual</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Architecture split added on 2026-06-30; current app ships settings/docs, not the Upgrade Transcript job itself.</t>
+          <t>Manual verification confirmed provider radios in Providers settings and provider submenus in overlay More-actions on 2026-06-30.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>SET-002</t>
+          <t>SET-010</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -3042,27 +3034,27 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Audio input selection</t>
+          <t>Unified provider settings</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to pick the microphone or virtual device RTI should use.</t>
+          <t>As a user, I want one settings surface for both provider selection and stored credentials so swapping models is simple.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Settings list system default plus available input devices, persist a preferred input UID, and apply it on the next session.</t>
+          <t>The Providers tab combines assistant-provider selection, STT-provider selection, and stored keys for all supported providers, with provider-specific missing-key guidance and no separate assistant/transcription provider sections in General. The Sessions Control workspace now exposes those settings pages directly in its main left rail instead of treating them as a nested settings-within-settings shell.</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; General</t>
+          <t>Sessions Control &gt; Providers / Modes / Prompts / Glossary / General; Settings command</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/AudioInputDevice.swift</t>
+          <t>RTI/Sources/Settings/SettingsView.swift; RTI/Sources/Settings/KeysTab.swift; RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/UI/SessionsControl/SessionsControlView.swift; RTI/Sources/UI/WindowCoordinator.swift</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3072,16 +3064,20 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>automated-pass</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
-      <c r="K52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Unified control navigation implemented 2026-06-30; `WindowCoordinator.openSettings()` now lands on the integrated Providers page in Sessions Control.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>SET-003</t>
+          <t>SET-011</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -3091,27 +3087,27 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Echo cancellation toggle</t>
+          <t>Async transcript-upgrade provider selection</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to optionally enable acoustic echo cancellation when I am on speakers.</t>
+          <t>As a user, I want a separate provider choice for future transcript upgrades so I can use a better batch provider than the live one.</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Settings persist an echo-cancellation preference, explain the current risk of silent microphones on some Macs, and apply the choice on the next session.</t>
+          <t>Providers settings distinguish `Real-time speech-to-text` from `Transcript upgrade (async)`, persist the async provider separately, and store any async-only credentials such as Aliyun without affecting the live lane.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Settings &gt; General</t>
+          <t>Settings &gt; Providers</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/AudioCaptureManager.swift</t>
+          <t>RTI/Sources/Soniox/SonioxClient.swift; RTI/Sources/Settings/KeysTab.swift; RTI/Sources/Settings/KeychainStore.swift; RTI/Sources/Secrets.swift</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3121,16 +3117,20 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>automated-pass</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
-      <c r="K53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Architecture split added on 2026-06-30; current app ships settings/docs, not the Upgrade Transcript job itself.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>SET-004</t>
+          <t>SET-002</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -3140,17 +3140,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Protect Bluetooth headphone volume</t>
+          <t>Audio input selection</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to avoid lowering my Bluetooth headphone volume during capture.</t>
+          <t>As a user, I want to pick the microphone or virtual device RTI should use.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Settings expose a persisted toggle that keeps Bluetooth headphones at full volume by favoring the built-in mic during recording and restoring the earlier mic on stop.</t>
+          <t>Settings list system default plus available input devices, persist a preferred input UID, and apply it on the next session.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/BluetoothMicGuard.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/AudioInputDevice.swift</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3179,7 +3179,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>SET-005</t>
+          <t>SET-003</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -3189,17 +3189,17 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Launch at login</t>
+          <t>Echo cancellation toggle</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to open automatically when I log into my Mac.</t>
+          <t>As a user, I want to optionally enable acoustic echo cancellation when I am on speakers.</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Settings reflect the current launch-at-login state, attempt to change it, and restore the previous toggle plus surface an error if the change fails.</t>
+          <t>Settings persist an echo-cancellation preference, explain the current risk of silent microphones on some Macs, and apply the choice on the next session.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Settings/LaunchAtLogin.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/AudioCaptureManager.swift</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3228,7 +3228,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>SET-006</t>
+          <t>SET-004</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -3238,17 +3238,17 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Audio monitor</t>
+          <t>Protect Bluetooth headphone volume</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to verify that RTI is capturing both my side and the other party before or during a meeting.</t>
+          <t>As a user, I want RTI to avoid lowering my Bluetooth headphone volume during capture.</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Settings embed a live audio monitor with current device and level information; the same monitor is also available from the menubar.</t>
+          <t>Settings expose a persisted toggle that keeps Bluetooth headphones at full volume by favoring the built-in mic during recording and restoring the earlier mic on stop.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/UI/AudioMonitor/AudioMonitorView.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Audio/BluetoothMicGuard.swift</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3277,7 +3277,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>SET-007</t>
+          <t>SET-005</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -3287,17 +3287,17 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Hotkey reference</t>
+          <t>Launch at login</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want a single place to confirm RTI's global shortcuts.</t>
+          <t>As a user, I want RTI to open automatically when I log into my Mac.</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Settings list the principal global hotkeys and explain that Command-Return is remappable while additional quick AI actions live in the command palette.</t>
+          <t>Settings reflect the current launch-at-login state, attempt to change it, and restore the previous toggle plus surface an error if the change fails.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/Settings/LaunchAtLogin.swift</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3326,7 +3326,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>SET-008</t>
+          <t>SET-006</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3336,17 +3336,17 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Data and support actions</t>
+          <t>Audio monitor</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want quick access to RTI's support folder, crash log, and logs.</t>
+          <t>As a user, I want to verify that RTI is capturing both my side and the other party before or during a meeting.</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Settings can reveal the RTI Application Support folder, reveal a crash log if one exists, and route to the logs viewer.</t>
+          <t>Settings embed a live audio monitor with current device and level information; the same monitor is also available from the menubar.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/GeneralTab.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift; RTI/Sources/UI/AudioMonitor/AudioMonitorView.swift</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3375,7 +3375,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>SET-009</t>
+          <t>SET-007</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3385,17 +3385,17 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Diagnostics copy</t>
+          <t>Hotkey reference</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to copy a concise diagnostics bundle for support or debugging.</t>
+          <t>As a user, I want a single place to confirm RTI's global shortcuts.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Settings surface version, model, and provider diagnostics and can copy a formatted diagnostics block to the pasteboard.</t>
+          <t>Settings list the principal global hotkeys and explain that Command-Return is remappable while additional quick AI actions live in the command palette.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -3424,37 +3424,37 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>DOC-001</t>
+          <t>SET-008</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Transcription lane documentation</t>
+          <t>Data and support actions</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>As a developer or operator, I want clear documentation for live transcription versus future transcript upgrades so provider choices are unambiguous.</t>
+          <t>As a user, I want quick access to RTI's support folder, crash log, and logs.</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Docs explain that real-time STT and async transcript upgrade are separate lanes, recommend provider defaults per laneand describe how the Upgrade Transcript action replaces the rough transcript.</t>
+          <t>Settings can reveal the RTI Application Support folder, reveal a crash log if one exists, and route to the logs viewer.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>README; docs</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>README.md; docs/transcript-upgrade-providers.md</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3464,50 +3464,46 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>automated-pass</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>Documentation added 2026-06-30 and tied to the transcribe skill’s provider defaults.</t>
-        </is>
-      </c>
+      <c r="K60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>LOG-001</t>
+          <t>SET-009</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Logs</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Live and past logs viewer</t>
+          <t>Diagnostics copy</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to inspect RTI's current and past application logs without opening files manually.</t>
+          <t>As a user, I want to copy a concise diagnostics bundle for support or debugging.</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>The logs window switches between live in-memory entries and past daily files, supports copy, clear or reveal actions appropriate to each mode, and shows the crash log in an expandable section.</t>
+          <t>Settings surface version, model, and provider diagnostics and can copy a formatted diagnostics block to the pasteboard.</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Sessions Control &gt; Logs</t>
+          <t>Settings &gt; General</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Settings/LogsView.swift; RTI/Sources/Support/AppLog.swift; RTI/Sources/Support/CrashLog.swift</t>
+          <t>RTI/Sources/Settings/GeneralTab.swift</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3517,50 +3513,46 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>passed-manual</t>
+          <t>not-tested</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>Manual smoke pass on 2026-06-30: verified live/past toggle, past-date selector, copy/reveal controls, and crash-log disclosure inside Sessions Control.</t>
-        </is>
-      </c>
+      <c r="K61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>ARC-001</t>
+          <t>DOC-001</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Archive</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Session archive browser</t>
+          <t>Transcription lane documentation</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to read past RTI sessions inside the app after they are saved.</t>
+          <t>As a developer or operator, I want clear documentation for live transcription versus future transcript upgrades so provider choices are unambiguous.</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>The Sessions browser loads recent archive folders, groups them by date buckets, opens a selected session, and defaults to the highest-priority available file.</t>
+          <t>Docs explain that real-time STT and async transcript upgrade are separate lanes, recommend provider defaults per laneand describe how the Upgrade Transcript action replaces the rough transcript.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Sessions window &gt; Sessions; notifications; overlay more menu</t>
+          <t>README; docs</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/SessionsControl/SessionsBrowserView.swift; RTI/Sources/Session/SessionArchive.swift; RTI/Sources/UI/WindowCoordinator.swift</t>
+          <t>README.md; docs/transcript-upgrade-providers.md</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -3570,46 +3562,50 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>automated-pass</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
-      <c r="K62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Documentation added 2026-06-30 and tied to the transcribe skill’s provider defaults.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>ARC-002</t>
+          <t>LOG-001</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Archive</t>
+          <t>Logs</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Session file copy and export</t>
+          <t>Live and past logs viewer</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want to copy or export archived session files for sharing or further work outside RTI.</t>
+          <t>As a user, I want to inspect RTI's current and past application logs without opening files manually.</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>The Sessions browser can copy the current markdown, export markdown, export PDF, and reveal the backing session folder in Finder.</t>
+          <t>The logs window switches between live in-memory entries and past daily files, supports copy, clear or reveal actions appropriate to each mode, and shows the crash log in an expandable section.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Sessions window &gt; Sessions</t>
+          <t>Sessions Control &gt; Logs</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/UI/SessionsControl/SessionsBrowserView.swift</t>
+          <t>RTI/Sources/Settings/LogsView.swift; RTI/Sources/Support/AppLog.swift; RTI/Sources/Support/CrashLog.swift</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -3619,16 +3615,20 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>not-tested</t>
+          <t>passed-manual</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
-      <c r="K63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Manual smoke pass on 2026-06-30: verified live/past toggle, past-date selector, copy/reveal controls, and crash-log disclosure inside Sessions Control.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>ARC-003</t>
+          <t>ARC-001</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -3638,27 +3638,27 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>End-of-session writeout</t>
+          <t>Session archive browser</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>As a user, I want RTI to preserve text artifacts from a finished session without keeping audio.</t>
+          <t>As a user, I want to read past RTI sessions inside the app after they are saved.</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>On stop, RTI can write transcript, chat, and screen-context artifacts into a timestamped session folder with owner-only permissions; live translation tokens are excluded from the kept transcript.</t>
+          <t>The Sessions browser loads recent archive folders, groups them by date buckets, opens a selected session, and defaults to the highest-priority available file.</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Implicit session lifecycle</t>
+          <t>Sessions window &gt; Sessions; notifications; overlay more menu</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>RTI/Sources/Session/SessionArchive.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
+          <t>RTI/Sources/UI/SessionsControl/SessionsBrowserView.swift; RTI/Sources/Session/SessionArchive.swift; RTI/Sources/UI/WindowCoordinator.swift</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3677,51 +3677,149 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
+          <t>ARC-002</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Archive</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Session file copy and export</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>As a user, I want to copy or export archived session files for sharing or further work outside RTI.</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>The Sessions browser can copy the current markdown, export markdown, export PDF, and reveal the backing session folder in Finder.</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Sessions window &gt; Sessions</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>RTI/Sources/UI/SessionsControl/SessionsBrowserView.swift</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>mapped</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>ARC-003</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Archive</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>End-of-session writeout</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>As a user, I want RTI to preserve text artifacts from a finished session without keeping audio.</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>On stop, RTI can write transcript, chat, notes, and screen-context artifacts into a timestamped session folder with owner-only permissions; live translation tokens are excluded from the kept transcript.</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Implicit session lifecycle</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>RTI/Sources/Session/SessionArchive.swift; RTI/Sources/Session/SessionCoordinator.swift</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>mapped</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>not-tested</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
           <t>ARC-005</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>Archive</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>Session-local retained audio</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>As a user, I want any retained session audio to live beside the transcript so the session folder is self-contained for upgrades and review.</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>When a session is archived, any kept `mic` and `system` `.m4a` files are moved into that session folder as `audio-mic.m4a` and `audio-system.m4a` on a best-effort basis.</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>Implicit session lifecycle</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>RTI/Sources/Session/SessionArchive.swift; RTI/Sources/Session/SessionCoordinator.swift; RTI/Sources/Audio/WAVWriter.swift</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
-        <is>
-          <t>mapped</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>mapped</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
         <is>
           <t>automated-pass</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr"/>
-      <c r="K65" s="2" t="inlineStr">
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr">
         <is>
           <t>Forward path implemented 2026-06-30; retroactive migration for old recordings remains to be done conservatively.</t>
         </is>
@@ -3774,8 +3872,10 @@
           <t>Inventory rows</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>64</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
       </c>
     </row>
     <row r="5">

</xml_diff>